<commit_message>
found issue, eq pot working
</commit_message>
<xml_diff>
--- a/Hardware/Design/Issue Log.xlsx
+++ b/Hardware/Design/Issue Log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indesignllc1-my.sharepoint.com/personal/adwolfe_indesign-llc_com/Documents/M_Drive/Github/Home-Audio-System/Hardware/Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_F25DC773A252ABDACC1048A061DA4FC05ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3C04EE6-37F3-4380-AE6B-09BBE114F8C8}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC1048A061DA4FC05ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{123B6086-87E4-4414-9D2C-9BAD61E890DC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>All input sources cannot be selected</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>pull up data lines to 3V3 and pull common down to ground</t>
+  </si>
+  <si>
+    <t>IC45 isn't getting 2.5V to pin 3</t>
   </si>
 </sst>
 </file>
@@ -382,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:E8"/>
+  <dimension ref="B3:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -474,6 +477,17 @@
         <v>11</v>
       </c>
     </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1">
+        <v>45860</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>